<commit_message>
Agregar nueva respuesta del cuestionario y excel actualizado
</commit_message>
<xml_diff>
--- a/02_Evidencias/Cuestionario/Respuestas/Respuestas_Cuestionario_MundiPets.xlsx
+++ b/02_Evidencias/Cuestionario/Respuestas/Respuestas_Cuestionario_MundiPets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy Mendoza\Music\MundiPets-PFC-IngReq\02_Evidencias\Cuestionario\Respuestas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B466D78E-24C8-46CF-B1BC-0B8170FADCA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D45D5F3-05C0-4D6C-9E95-F9B148FE1CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="158">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -484,6 +484,18 @@
   </si>
   <si>
     <t xml:space="preserve">Es indispensable conocer el estado de salud de ambos gatos salud vacunas enfermedades hereditarias y asegurarse que la cruza sea responsable y beneficie el bienestar de los animales </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La flta de información </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Información de temas como la importancia de saber que razas pueden o no cruzarse </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguridad de que sera una prioridad en el hogar </t>
+  </si>
+  <si>
+    <t>No lo se</t>
   </si>
 </sst>
 </file>
@@ -608,7 +620,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:S38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:S39">
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Marca temporal"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="1. Tipo de usuario "/>
@@ -835,7 +847,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18.88671875" customWidth="1"/>
@@ -3047,6 +3059,65 @@
         <v>153</v>
       </c>
     </row>
+    <row r="39" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>46231.391812523143</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="3">
+        <v>5</v>
+      </c>
+      <c r="E39" s="3">
+        <v>4</v>
+      </c>
+      <c r="F39" s="3">
+        <v>5</v>
+      </c>
+      <c r="G39" s="3">
+        <v>5</v>
+      </c>
+      <c r="H39" s="3">
+        <v>5</v>
+      </c>
+      <c r="I39" s="3">
+        <v>3</v>
+      </c>
+      <c r="J39" s="3">
+        <v>4</v>
+      </c>
+      <c r="K39" s="3">
+        <v>4</v>
+      </c>
+      <c r="L39" s="3">
+        <v>4</v>
+      </c>
+      <c r="M39" s="3">
+        <v>4</v>
+      </c>
+      <c r="N39" s="3">
+        <v>4</v>
+      </c>
+      <c r="O39" s="3">
+        <v>3</v>
+      </c>
+      <c r="P39" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q39" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="R39" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="S39" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>